<commit_message>
fix: Excel 계산 예시 오류 수정 + REPLACE vs STACK 구분 명시
오류 수정:
- 31_CALC_Example_SKT: 혜택가 18,300원 → 23,800원 (5,500원 오류 수정)
- 원인: 요즘가족결합을 요즘우리집 REPLACE 방식이 아니라 추가 할인으로 잘못 계산
- 정답: 단독가(33,000) 기준으로 재계산 (tvInternetNoWifi 무시)

추가 시트:
- 31b_CALC_Example_KT_Total: KT 총액결합 STACK 방식 예시
  (기본 TV결합 할인 + 총액할인 중복 적용)

30_CALC_Formula 시트 강화:
- ⚠️ 3사 결합할인 적용 방식 차이 주의사항 명시
  · SKT 요즘가족: REPLACE
  · KT 총액/정액: STACK
  · KT 프리미엄: 대표자/프리미엄 대상 독립 계산
  · LGU+ 참쉬운/투게더: REPLACE

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bongi-calculator-data.xlsx
+++ b/docs/bongi-calculator-data.xlsx
@@ -24,8 +24,9 @@
     <sheet name="15_LGU_Together" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="30_CALC_Formula" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="31_CALC_Example_SKT" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="32_CALC_Example_KT_Premium" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="20_Schema" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="31b_CALC_Example_KT_Total" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="32_CALC_Example_KT_Premium" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="20_Schema" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,6 +131,12 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Noto Sans KR"/>
+      <b val="1"/>
+      <color rgb="00dc2626"/>
+      <sz val="13"/>
+    </font>
+    <font>
       <name val="SF Mono"/>
       <sz val="10"/>
     </font>
@@ -219,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -257,27 +264,30 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2475,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2653,304 +2663,354 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>⚠️ 핵심 주의사항 — 3사 결합할인 적용 방식 다름</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>• SKT 요즘가족결합: 단독가 **REPLACE** (요즘우리집 대체) → tvInternetNoWifi 무시</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>• KT 총액/정액: 기본 TV결합할인 + 총액할인 **STACK** (중복 적용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>• KT 프리미엄: 총액대상(대표자+77K미만) + 프리미엄대상(77K↑) 독립 계산</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>• LG U+ 참쉬운: 단독가 **REPLACE** (SKT와 유사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>• LG U+ 투게더: 단독가 **REPLACE** (85K↑ 고가요금제 한정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>🏷️ 결합할인 계산 — 통신사별 분기</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>통신사</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>결합 종류</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>계산 공식</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t>SKT</t>
         </is>
       </c>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>요즘가족결합</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C31" s="28" t="inlineStr">
         <is>
           <t>inetDc = D.skt.bundle.family.internet[sp]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="inlineStr"/>
-      <c r="B24" s="24" t="inlineStr"/>
-      <c r="C24" s="27" t="inlineStr">
-        <is>
-          <t>iptvDc = hasTv ? D.skt.bundle.family.iptv : 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="24" t="inlineStr"/>
-      <c r="B25" s="24" t="inlineStr"/>
-      <c r="C25" s="27" t="inlineStr">
-        <is>
-          <t>mobPer = D.skt.bundle.family.mobilePerBySpeed[sp][lines]</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr"/>
-      <c r="B26" s="24" t="inlineStr"/>
-      <c r="C26" s="27" t="inlineStr">
-        <is>
-          <t>mobTotal = mobPer × lines  ← 인당 × 인원</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr"/>
-      <c r="B27" s="24" t="inlineStr"/>
-      <c r="C27" s="27" t="inlineStr">
-        <is>
-          <t>bundleDc = inetDc + iptvDc (인터넷/TV 할인)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="24" t="inlineStr"/>
-      <c r="B28" s="24" t="inlineStr"/>
-      <c r="C28" s="27" t="inlineStr">
-        <is>
-          <t>mobileSideDiscount = mobTotal (휴대폰 고지서에서 별도 차감)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="B29" s="28" t="inlineStr">
-        <is>
-          <t>총액결합 (total)</t>
-        </is>
-      </c>
-      <c r="C29" s="29" t="inlineStr">
-        <is>
-          <t>rngIdx = 합산_요금_구간 (6단계)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="24" t="inlineStr"/>
-      <c r="B30" s="24" t="inlineStr"/>
-      <c r="C30" s="27" t="inlineStr">
-        <is>
-          <t>inetDc = D.kt.bundle.total.internet[sp][rngIdx]</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="24" t="inlineStr"/>
-      <c r="B31" s="24" t="inlineStr"/>
-      <c r="C31" s="27" t="inlineStr">
-        <is>
-          <t>mobDc = D.kt.bundle.total.mobile[sp][rngIdx]</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="inlineStr"/>
       <c r="B32" s="24" t="inlineStr"/>
-      <c r="C32" s="27" t="inlineStr">
-        <is>
-          <t>bundleDc = inetDc (인터넷 할인 · 기본 TV결합할인과 중복 적용)</t>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>iptvDc = hasTv ? D.skt.bundle.family.iptv : 0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr"/>
       <c r="B33" s="24" t="inlineStr"/>
-      <c r="C33" s="27" t="inlineStr">
-        <is>
-          <t>mobileSideDiscount = mobDc</t>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>mobPer = D.skt.bundle.family.mobilePerBySpeed[sp][lines]</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>정액결합 (fixed)</t>
-        </is>
-      </c>
+      <c r="A34" s="24" t="inlineStr"/>
+      <c r="B34" s="24" t="inlineStr"/>
       <c r="C34" s="29" t="inlineStr">
         <is>
-          <t>fxIdx = 요금_구간 (4단계)</t>
+          <t>mobTotal = mobPer × lines  ← 인당 × 인원</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr"/>
       <c r="B35" s="24" t="inlineStr"/>
-      <c r="C35" s="27" t="inlineStr">
-        <is>
-          <t>inetDc = D.kt.bundle.fixed.internet[fxIdx]  (전구간 5,500)</t>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>bundleDc = inetDc + iptvDc (인터넷/TV 할인)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr"/>
       <c r="B36" s="24" t="inlineStr"/>
-      <c r="C36" s="27" t="inlineStr">
-        <is>
-          <t>mobDc = D.kt.bundle.fixed.mobile[fxIdx]</t>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>mobileSideDiscount = mobTotal (휴대폰 고지서에서 별도 차감)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="28" t="inlineStr">
+      <c r="A37" s="30" t="inlineStr">
         <is>
           <t>KT</t>
         </is>
       </c>
-      <c r="B37" s="28" t="inlineStr">
-        <is>
-          <t>💎 프리미엄 가족결합</t>
-        </is>
-      </c>
-      <c r="C37" s="29" t="inlineStr">
-        <is>
-          <t>자격: 77K↑ 요금제 2회선 이상</t>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>총액결합 (total)</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>rngIdx = 합산_요금_구간 (6단계)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="24" t="inlineStr"/>
       <c r="B38" s="24" t="inlineStr"/>
-      <c r="C38" s="27" t="inlineStr">
-        <is>
-          <t>대표자 + 77K미만 구성원 → 총액결합 합산 → 구간 mobDc</t>
+      <c r="C38" s="29" t="inlineStr">
+        <is>
+          <t>inetDc = D.kt.bundle.total.internet[sp][rngIdx]</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="24" t="inlineStr"/>
       <c r="B39" s="24" t="inlineStr"/>
-      <c r="C39" s="27" t="inlineStr">
-        <is>
-          <t>77K↑ 구성원(대표자 제외) → 각각 D.kt.bundle.premium.planCatalog[plan].dc 합산</t>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>mobDc = D.kt.bundle.total.mobile[sp][rngIdx]</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="24" t="inlineStr"/>
       <c r="B40" s="24" t="inlineStr"/>
-      <c r="C40" s="27" t="inlineStr">
-        <is>
-          <t>totalDc = 5500 (인터넷 고정) + 총액결합mobDc + 프리미엄dc 합</t>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>bundleDc = inetDc (인터넷 할인 · 기본 TV결합할인과 중복 적용)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>LG U+</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>참쉬운가족결합</t>
-        </is>
-      </c>
-      <c r="C41" s="31" t="inlineStr">
-        <is>
-          <t>inetDc = D.lgu.bundle.chweyswun.internet[sp]</t>
+      <c r="A41" s="24" t="inlineStr"/>
+      <c r="B41" s="24" t="inlineStr"/>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>mobileSideDiscount = mobDc</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr"/>
-      <c r="B42" s="24" t="inlineStr"/>
-      <c r="C42" s="27" t="inlineStr">
-        <is>
-          <t>planIdx = 요금제_구간 (3단계: 69K미만/69K↑/88K↑)</t>
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>정액결합 (fixed)</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>fxIdx = 요금_구간 (4단계)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="24" t="inlineStr"/>
       <c r="B43" s="24" t="inlineStr"/>
-      <c r="C43" s="27" t="inlineStr">
-        <is>
-          <t>lineIdx = min(lines,4) - 2  ← 2회선:0, 3회선:1, 4+:2</t>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>inetDc = D.kt.bundle.fixed.internet[fxIdx]  (전구간 5,500)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="24" t="inlineStr"/>
       <c r="B44" s="24" t="inlineStr"/>
-      <c r="C44" s="27" t="inlineStr">
-        <is>
-          <t>mobDc = D.lgu.bundle.chweyswun.mobile[planIdx][lineIdx]</t>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>mobDc = D.kt.bundle.fixed.mobile[fxIdx]</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="30" t="inlineStr">
         <is>
-          <t>LG U+</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B45" s="30" t="inlineStr">
         <is>
-          <t>투게더 결합</t>
+          <t>💎 프리미엄 가족결합</t>
         </is>
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>자격: 85K↑ 고가요금제 (100M 결합 불가)</t>
+          <t>자격: 77K↑ 요금제 2회선 이상</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr"/>
       <c r="B46" s="24" t="inlineStr"/>
-      <c r="C46" s="27" t="inlineStr">
-        <is>
-          <t>inetDc = D.lgu.bundle.together.internet[sp]  (100M=0)</t>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>대표자 + 77K미만 구성원 → 총액결합 합산 → 구간 mobDc</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="24" t="inlineStr"/>
       <c r="B47" s="24" t="inlineStr"/>
-      <c r="C47" s="27" t="inlineStr">
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>77K↑ 구성원(대표자 제외) → 각각 D.kt.bundle.premium.planCatalog[plan].dc 합산</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr"/>
+      <c r="B48" s="24" t="inlineStr"/>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>totalDc = 5500 (인터넷 고정) + 총액결합mobDc + 프리미엄dc 합</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>참쉬운가족결합</t>
+        </is>
+      </c>
+      <c r="C49" s="33" t="inlineStr">
+        <is>
+          <t>inetDc = D.lgu.bundle.chweyswun.internet[sp]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr"/>
+      <c r="B50" s="24" t="inlineStr"/>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
+          <t>planIdx = 요금제_구간 (3단계: 69K미만/69K↑/88K↑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr"/>
+      <c r="B51" s="24" t="inlineStr"/>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>lineIdx = min(lines,4) - 2  ← 2회선:0, 3회선:1, 4+:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr"/>
+      <c r="B52" s="24" t="inlineStr"/>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>mobDc = D.lgu.bundle.chweyswun.mobile[planIdx][lineIdx]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="inlineStr">
+        <is>
+          <t>투게더 결합</t>
+        </is>
+      </c>
+      <c r="C53" s="33" t="inlineStr">
+        <is>
+          <t>자격: 85K↑ 고가요금제 (100M 결합 불가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="inlineStr"/>
+      <c r="B54" s="24" t="inlineStr"/>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>inetDc = D.lgu.bundle.together.internet[sp]  (100M=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="inlineStr"/>
+      <c r="B55" s="24" t="inlineStr"/>
+      <c r="C55" s="29" t="inlineStr">
         <is>
           <t>mobDc = D.lgu.bundle.together.mobile[lineIdx]</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A22:B22"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2961,7 +3021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2977,355 +3037,507 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="34" t="inlineStr">
         <is>
           <t>입력값</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr"/>
-      <c r="C3" s="33" t="inlineStr"/>
+      <c r="B3" s="29" t="inlineStr"/>
+      <c r="C3" s="35" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="34" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  통신사</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>SKT</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C4" s="35" t="inlineStr">
         <is>
           <t>D["skt"]</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  속도</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>500M</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr"/>
+      <c r="C5" s="35" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  TV 상품</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>B tv 올 (tvIdx=3)</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>D.skt.tv[3] = {p:18700, dc:2200}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  WiFi</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>없음</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr"/>
+      <c r="C7" s="35" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  결합 종류</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>요즘가족결합 (family)</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr"/>
+      <c r="C8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  결합 인원</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>3명</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr"/>
+      <c r="C9" s="35" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="35" t="inlineStr"/>
-      <c r="B10" s="36" t="inlineStr"/>
-      <c r="C10" s="37" t="inlineStr"/>
+      <c r="A10" s="37" t="inlineStr"/>
+      <c r="B10" s="38" t="inlineStr"/>
+      <c r="C10" s="39" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
-        <is>
-          <t>기본가 계산</t>
-        </is>
-      </c>
-      <c r="B11" s="27" t="inlineStr"/>
-      <c r="C11" s="33" t="inlineStr"/>
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>【경로 A】 휴대폰 결합 X (요즘우리집결합만 적용)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr"/>
+      <c r="C11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. 인터넷 결합가 (WiFi 미포함)</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. 인터넷 결합가 (tvInternetNoWifi)</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>27,500원</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="35" t="inlineStr">
         <is>
           <t>D.skt.tvInternetNoWifi["500M"]</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. TV 최종요금 (결합할인 후)</t>
-        </is>
-      </c>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. TV 최종요금 (결합할인 -2,200)</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>16,500원</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>18,700 - 2,200</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  3. 셋톱박스 스마트3</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>4,400원</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>D.skt.setTopOptions[0].fee</t>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>D.skt.setTop</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  = 월 기본요금</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = 월 기본요금 (요즘우리집)</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>48,400원</t>
         </is>
       </c>
-      <c r="C15" s="39" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>27,500 + 16,500 + 4,400</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="35" t="inlineStr"/>
-      <c r="B16" s="36" t="inlineStr"/>
-      <c r="C16" s="37" t="inlineStr"/>
+      <c r="A16" s="37" t="inlineStr"/>
+      <c r="B16" s="38" t="inlineStr"/>
+      <c r="C16" s="39" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="32" t="inlineStr">
-        <is>
-          <t>요즘가족결합 할인</t>
-        </is>
-      </c>
-      <c r="B17" s="27" t="inlineStr"/>
-      <c r="C17" s="33" t="inlineStr"/>
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>【경로 B】 휴대폰 결합 O (요즘가족결합 적용 · 요즘우리집 REPLACE)</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr"/>
+      <c r="C17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  인터넷 할인</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ※ 주의: 단독가에서 재계산 (tvInternetNoWifi 사용 X)</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr"/>
+      <c r="C18" s="35" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. 인터넷 단독가 500M</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>33,000원</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>D.skt.internet["500M"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. 요즘가족결합 인터넷 할인</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t>-11,000원</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C20" s="35" t="inlineStr">
         <is>
           <t>D.skt.bundle.family.internet["500M"]</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  IPTV 추가 할인 (TV 결합 시)</t>
-        </is>
-      </c>
-      <c r="B19" s="27" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → 인터넷 실질</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>22,000원</t>
+        </is>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>33,000 - 11,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. TV 기본 (B tv 올)</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>18,700원</t>
+        </is>
+      </c>
+      <c r="C22" s="35" t="inlineStr">
+        <is>
+          <t>D.skt.tv[3].p</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. TV 결합할인</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>-2,200원</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>D.skt.tv[3].dc</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. IPTV 추가 할인 (요즘가족 전용)</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
         <is>
           <t>-1,100원</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>D.skt.bundle.family.iptv</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  휴대폰 할인 (500M, 3회선 × 6,000)</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>-18,000원</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="inlineStr">
-        <is>
-          <t>mobilePerBySpeed["500M"][3] × 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="35" t="inlineStr"/>
-      <c r="B21" s="36" t="inlineStr"/>
-      <c r="C21" s="37" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>최종 계산</t>
-        </is>
-      </c>
-      <c r="B22" s="27" t="inlineStr"/>
-      <c r="C22" s="33" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  인터넷+TV 실납부</t>
-        </is>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>36,300원</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>48,400 - 11,000 - 1,100</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  휴대폰 고지서 별도 차감</t>
-        </is>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>-18,000원</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="inlineStr">
-        <is>
-          <t>(3회선 합산)</t>
-        </is>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🎉 혜택가 (최종)</t>
-        </is>
-      </c>
-      <c r="B25" s="26" t="inlineStr">
-        <is>
-          <t>18,300원/월</t>
-        </is>
-      </c>
-      <c r="C25" s="39" t="inlineStr">
-        <is>
-          <t>36,300 - 18,000</t>
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → TV 실질</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>15,400원</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>18,700 - 2,200 - 1,100</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="35" t="inlineStr"/>
-      <c r="B26" s="36" t="inlineStr"/>
-      <c r="C26" s="37" t="inlineStr"/>
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  6. 셋톱박스</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>4,400원</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
-        <is>
-          <t>부가 혜택</t>
-        </is>
-      </c>
-      <c r="B27" s="27" t="inlineStr"/>
-      <c r="C27" s="33" t="inlineStr"/>
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = 인터넷+TV 월 실납부</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>41,800원</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="inlineStr">
+        <is>
+          <t>22,000 + 15,400 + 4,400</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  설치비 (1회성)</t>
-        </is>
-      </c>
-      <c r="B28" s="27" t="inlineStr">
-        <is>
-          <t>56,100원</t>
-        </is>
-      </c>
-      <c r="C28" s="33" t="inlineStr">
-        <is>
-          <t>D.skt.install.combo</t>
-        </is>
-      </c>
+      <c r="A28" s="37" t="inlineStr"/>
+      <c r="B28" s="38" t="inlineStr"/>
+      <c r="C28" s="39" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="34" t="inlineStr">
         <is>
+          <t>휴대폰 고지서 별도 차감</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr"/>
+      <c r="C29" s="35" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  휴대폰 할인 인당 (500M, 3회선)</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>6,000원</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>mobilePerBySpeed["500M"][3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  총 할인 (인당 × 회선수)</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>-18,000원</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="inlineStr">
+        <is>
+          <t>6,000 × 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="37" t="inlineStr"/>
+      <c r="B32" s="38" t="inlineStr"/>
+      <c r="C32" s="39" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎉 혜택가 (최종)</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>23,800원/월</t>
+        </is>
+      </c>
+      <c r="C33" s="41" t="inlineStr">
+        <is>
+          <t>41,800 - 18,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="37" t="inlineStr"/>
+      <c r="B34" s="38" t="inlineStr"/>
+      <c r="C34" s="39" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>경로 A vs B 차이</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="inlineStr"/>
+      <c r="C35" s="35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  요즘우리집 (A): 48,400원</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr"/>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>휴대폰 결합 없을 때</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  요즘가족 (B): 23,800원</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="inlineStr"/>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>휴대폰 3회선 결합 시 (-24,600 절감)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="37" t="inlineStr"/>
+      <c r="B38" s="38" t="inlineStr"/>
+      <c r="C38" s="39" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>부가 혜택</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr"/>
+      <c r="C39" s="35" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  설치비 (1회성, 결합)</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>56,100원</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="inlineStr">
+        <is>
+          <t>D.skt.install.combo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="36" t="inlineStr">
+        <is>
           <t xml:space="preserve">  사은품 (500M + TV 결합)</t>
         </is>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B41" s="29" t="inlineStr">
         <is>
           <t>430,000원</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C41" s="35" t="inlineStr">
         <is>
           <t>D.skt.gift.combo["500M"]</t>
         </is>
@@ -3337,6 +3549,425 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>🧮 KT 총액결합 계산 예시 — 500M+지니TV 에센스+WiFi O+총액결합(108,900원↑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>입력값</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr"/>
+      <c r="C3" s="35" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  통신사/속도</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>KT 500M</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TV 상품</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>지니TV 에센스 (tvIdx=3)</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.tv[3] = {p:20240, dc:3740}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WiFi</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>사용 (+1,100원)</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.wifiPrice["500M"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  결합 종류</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>총액결합 (kt-total)</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  휴대폰 합산 구간</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>108,900원 이상 (rngIdx=3)</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="inlineStr"/>
+      <c r="B9" s="29" t="inlineStr"/>
+      <c r="C9" s="35" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>【기본 TV 결합 인터넷 할인】 (KT 기본)</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr"/>
+      <c r="C10" s="35" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  인터넷 단독 (500M)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>33,000원</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.internet["500M"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WiFi 추가</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>+1,100원</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  인터넷 결합가 (tvInternetWithWifi)</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>28,600원</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.tvInternetWithWifi["500M"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → 기본 TV결합 인터넷 할인</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>-5,500원</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>(33,000+1,100) - 28,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr"/>
+      <c r="B15" s="29" t="inlineStr"/>
+      <c r="C15" s="35" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>【총액결합 추가 할인】 ← 중복 적용</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr"/>
+      <c r="C16" s="35" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  총액결합 인터넷 할인</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>-5,500원</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.bundle.total.internet["500M"][3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → 인터넷 최종</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>23,100원</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>28,600 - 5,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr"/>
+      <c r="B19" s="29" t="inlineStr"/>
+      <c r="C19" s="35" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>【TV + 셋톱】</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr"/>
+      <c r="C20" s="35" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TV 기본</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>20,240원</t>
+        </is>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.tv[3].p</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TV 결합할인</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>-3,740원</t>
+        </is>
+      </c>
+      <c r="C22" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.tv[3].dc</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → TV 실질</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>16,500원</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>20,240 - 3,740</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  셋톱박스 기가지니3</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>4,400원</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.setTop</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="inlineStr"/>
+      <c r="B25" s="29" t="inlineStr"/>
+      <c r="C25" s="35" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>【월 실납부】</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr"/>
+      <c r="C26" s="44" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  인터넷+TV+셋톱</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>44,000원</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="inlineStr">
+        <is>
+          <t>23,100 + 16,500 + 4,400</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr"/>
+      <c r="B28" s="29" t="inlineStr"/>
+      <c r="C28" s="35" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="34" t="inlineStr">
+        <is>
+          <t>휴대폰 고지서 별도 할인</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr"/>
+      <c r="C29" s="35" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  500M mobile[3]</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>-16,610원</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>D.kt.bundle.total.mobile["500M"][3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr"/>
+      <c r="B31" s="29" t="inlineStr"/>
+      <c r="C31" s="35" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎉 총 월 절감액 (vs 단독)</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>44,000 + (-16,610) 별도</t>
+        </is>
+      </c>
+      <c r="C32" s="44" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="42" t="inlineStr"/>
+      <c r="B33" s="29" t="inlineStr"/>
+      <c r="C33" s="35" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="34" t="inlineStr">
+        <is>
+          <t>※ KT 특성: 기본 TV결합 할인 + 총액결합 할인 **중복 적용** (STACK)</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="inlineStr"/>
+      <c r="C34" s="35" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   → SKT 요즘가족결합(REPLACE)과 반대 방식</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="inlineStr"/>
+      <c r="C35" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3358,597 +3989,227 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="34" t="inlineStr">
         <is>
           <t>입력값</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr"/>
-      <c r="C3" s="33" t="inlineStr"/>
+      <c r="B3" s="29" t="inlineStr"/>
+      <c r="C3" s="35" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  인터넷</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>100M + WiFi 없음 (TV 없음)</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr"/>
+      <c r="C4" s="35" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="40" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  회선 구성</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>대표 89K + 구성원 89K(프리미엄) + 구성원 89K(프리미엄)</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="35" t="inlineStr">
         <is>
           <t>총 3회선</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  총액결합 대상</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>대표자 89K만 (프리미엄 2명 제외)</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>합산 89,000원</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  구간 판정</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>64,900원 이상 (index 2)</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr"/>
+      <c r="C7" s="35" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr"/>
-      <c r="B8" s="27" t="inlineStr"/>
-      <c r="C8" s="33" t="inlineStr"/>
+      <c r="A8" s="42" t="inlineStr"/>
+      <c r="B8" s="29" t="inlineStr"/>
+      <c r="C8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>총액결합 할인 (대표자 몫)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr"/>
-      <c r="C9" s="33" t="inlineStr"/>
+      <c r="B9" s="29" t="inlineStr"/>
+      <c r="C9" s="35" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  100M mobile[index 2]</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>-3,300원</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="35" t="inlineStr">
         <is>
           <t>D.kt.bundle.total.mobile["100M"][2]</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="40" t="inlineStr"/>
-      <c r="B11" s="27" t="inlineStr"/>
-      <c r="C11" s="33" t="inlineStr"/>
+      <c r="A11" s="42" t="inlineStr"/>
+      <c r="B11" s="29" t="inlineStr"/>
+      <c r="C11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>프리미엄 할인 (구성원 2명)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="inlineStr"/>
-      <c r="C12" s="33" t="inlineStr"/>
+      <c r="B12" s="29" t="inlineStr"/>
+      <c r="C12" s="35" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="40" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  89,000원 요금제 × 25% (정확)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>-22,250원 × 2 = -44,500원</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>planCatalog[89000].dc</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="inlineStr"/>
-      <c r="B14" s="27" t="inlineStr"/>
-      <c r="C14" s="33" t="inlineStr"/>
+      <c r="A14" s="42" t="inlineStr"/>
+      <c r="B14" s="29" t="inlineStr"/>
+      <c r="C14" s="35" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="34" t="inlineStr">
         <is>
           <t>인터넷 할인 (고정)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="inlineStr"/>
-      <c r="C15" s="33" t="inlineStr"/>
+      <c r="B15" s="29" t="inlineStr"/>
+      <c r="C15" s="35" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="40" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  프리미엄 인터넷 할인</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>-5,500원</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="35" t="inlineStr">
         <is>
           <t>D.kt.bundle.premium.internet</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="40" t="inlineStr"/>
-      <c r="B17" s="27" t="inlineStr"/>
-      <c r="C17" s="33" t="inlineStr"/>
+      <c r="A17" s="42" t="inlineStr"/>
+      <c r="B17" s="29" t="inlineStr"/>
+      <c r="C17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="34" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr"/>
-      <c r="C18" s="33" t="inlineStr"/>
+      <c r="B18" s="29" t="inlineStr"/>
+      <c r="C18" s="35" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="45" t="inlineStr">
         <is>
           <t xml:space="preserve">  총 할인액</t>
         </is>
       </c>
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>-53,300원</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="44" t="inlineStr">
         <is>
           <t>3,300 + 44,500 + 5,500</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="40" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  총액결합만 했을 때 비교</t>
         </is>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t>-28,600원</t>
         </is>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" s="35" t="inlineStr">
         <is>
           <t>(174,900↑ 구간 기준)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  💎 프리미엄 선택 시 추가 이득</t>
-        </is>
-      </c>
-      <c r="B21" s="44" t="inlineStr">
-        <is>
-          <t>+24,700원 더 할인</t>
-        </is>
-      </c>
-      <c r="C21" s="45" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A56"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>📐 D 객체 JSON 스키마 (TypeScript 인터페이스)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="46" t="inlineStr">
-        <is>
-          <t>interface CarrierData {</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  name: string;          // "SKT (B tv)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  prefix: string;        // "SK" | "KT" | "LG"</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  wifiCost?: number;     // SKT, LGU+ 사용 (단일값)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  wifiPrice?: Record&lt;"100M"|"500M"|"1G", number&gt;;  // KT 사용 (속도별)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  setTopOptions: SetTop[];</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  wifiOptions: WiFi[];</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  tvInternetNoWifi: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  tvInternetWithWifi: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  tv: TVProduct[];</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  install: { solo: number; combo: number; };</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  gift: { solo: SpeedMap; combo: SpeedMap; };</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  bundle: BundleConfig;  // 통신사별 상이</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="46" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="46" t="inlineStr">
-        <is>
-          <t>interface SetTop { id: string; name: string; fee: number; isDefault?: boolean; active: boolean; }</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="46" t="inlineStr">
-        <is>
-          <t>interface WiFi { id: string; name: string; fees: Record&lt;"100M"|"500M"|"1G", number&gt;; isDefault?: boolean; active: boolean; }</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="46" t="inlineStr">
         <is>
-          <t>interface TVProduct { n: string; p: number; dc: number; }  // n=이름, p=단독가, dc=결합할인</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="46" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="46" t="inlineStr">
-        <is>
-          <t>type BundleConfig =</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  | { family: SktFamily }                              // SKT</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  | { ranges_total, total, ranges_fixed, fixed, premium }  // KT</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  | { chweyswun, together };                           // LGU+</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="46" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="46" t="inlineStr">
-        <is>
-          <t>interface SktFamily {</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: SpeedMap;</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  iptv: number;  // 1100</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mobilePerBySpeed: Record&lt;Speed, Record&lt;1|2|3|4|5, number&gt;&gt;;</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="46" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="46" t="inlineStr">
-        <is>
-          <t>interface KTTotal {</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: Record&lt;Speed, number[]&gt;;  // 6구간</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mobile: Record&lt;Speed, number[]&gt;;    // 6구간</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="46" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="46" t="inlineStr">
-        <is>
-          <t>interface KTPremium {</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: 5500;</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  planCatalog: Array&lt;{ v: number; label: string; dc: number; prem: boolean }&gt;;</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="46" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="46" t="inlineStr">
-        <is>
-          <t>interface LguChweyswun {</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: SpeedMap;</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  planLabels: string[];  // 3개</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mobile: number[][];    // 3 (요금구간) × 3 (회선수)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="46" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="46" t="inlineStr">
-        <is>
-          <t>interface LguTogether {</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  internet: SpeedMap;  // 100M=0 (불가)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mobile: [number, number, number];  // 2/3/4+회선</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="46" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="46" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="46" t="inlineStr">
-        <is>
-          <t>type Speed = "100M" | "500M" | "1G";</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="46" t="inlineStr">
-        <is>
-          <t>type SpeedMap = Record&lt;Speed, number&gt;;</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  💎 프리미엄 선택 시 추가 이득</t>
+        </is>
+      </c>
+      <c r="B21" s="47" t="inlineStr">
+        <is>
+          <t>+24,700원 더 할인</t>
+        </is>
+      </c>
+      <c r="C21" s="48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4072,6 +4333,376 @@
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>※ 3사 모두 3년 약정 기준 · 부가세 포함 · WiFi/셋톱 별도</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>📐 D 객체 JSON 스키마 (TypeScript 인터페이스)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="49" t="inlineStr">
+        <is>
+          <t>interface CarrierData {</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  name: string;          // "SKT (B tv)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  prefix: string;        // "SK" | "KT" | "LG"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  wifiCost?: number;     // SKT, LGU+ 사용 (단일값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  wifiPrice?: Record&lt;"100M"|"500M"|"1G", number&gt;;  // KT 사용 (속도별)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  setTopOptions: SetTop[];</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  wifiOptions: WiFi[];</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  tvInternetNoWifi: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  tvInternetWithWifi: Record&lt;"100M"|"500M"|"1G", number&gt;;</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  tv: TVProduct[];</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  install: { solo: number; combo: number; };</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gift: { solo: SpeedMap; combo: SpeedMap; };</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bundle: BundleConfig;  // 통신사별 상이</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>interface SetTop { id: string; name: string; fee: number; isDefault?: boolean; active: boolean; }</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>interface WiFi { id: string; name: string; fees: Record&lt;"100M"|"500M"|"1G", number&gt;; isDefault?: boolean; active: boolean; }</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>interface TVProduct { n: string; p: number; dc: number; }  // n=이름, p=단독가, dc=결합할인</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>type BundleConfig =</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  | { family: SktFamily }                              // SKT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  | { ranges_total, total, ranges_fixed, fixed, premium }  // KT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  | { chweyswun, together };                           // LGU+</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>interface SktFamily {</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: SpeedMap;</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  iptv: number;  // 1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mobilePerBySpeed: Record&lt;Speed, Record&lt;1|2|3|4|5, number&gt;&gt;;</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>interface KTTotal {</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: Record&lt;Speed, number[]&gt;;  // 6구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mobile: Record&lt;Speed, number[]&gt;;    // 6구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>interface KTPremium {</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: 5500;</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  planCatalog: Array&lt;{ v: number; label: string; dc: number; prem: boolean }&gt;;</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="49" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>interface LguChweyswun {</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: SpeedMap;</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  planLabels: string[];  // 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mobile: number[][];    // 3 (요금구간) × 3 (회선수)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>interface LguTogether {</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  internet: SpeedMap;  // 100M=0 (불가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mobile: [number, number, number];  // 2/3/4+회선</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="49" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="49" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="49" t="inlineStr">
+        <is>
+          <t>type Speed = "100M" | "500M" | "1G";</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="49" t="inlineStr">
+        <is>
+          <t>type SpeedMap = Record&lt;Speed, number&gt;;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: INDEX 참고자료에 calculator-v2.html 추가
- v1 (원본·상담원용 상세) + v2 (고객용·심플 카드형) 둘 다 링크
- 개발자가 v1/v2 차이와 용도 한눈에 파악 가능
- Excel 임시 lock 파일 정리

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bongi-calculator-data.xlsx
+++ b/docs/bongi-calculator-data.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1267,7 +1267,7 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>🔗 봉이모바일 통합 계산기 (원본 데이터 소스)</t>
+          <t>🔗 봉이모바일 통합 계산기 v1 (원본 · 상담원용 상세)</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -1279,17 +1279,29 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
+          <t>🔗 봉이모바일 계산기 v2 (고객용 · 심플 카드형 UI)</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>https://bongi-mobile-production.up.railway.app/docs/calculator-v2.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
           <t>🔗 GitHub 리포지토리</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>https://github.com/vinsenzo83/bongi-mobile</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="B38:C38"/>
@@ -1297,6 +1309,7 @@
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B41:C41"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="A35:C35"/>
@@ -1310,6 +1323,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(policy): 사은품 정책 카탈로그 (63개) - 엑셀 07_Gift_Catalog 시트 + flow-internet-tv 표 섹션
</commit_message>
<xml_diff>
--- a/docs/bongi-calculator-data.xlsx
+++ b/docs/bongi-calculator-data.xlsx
@@ -27,6 +27,7 @@
     <sheet name="15_LGU_Together" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="20_Schema" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="30_Formula" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="07_Gift_Catalog" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,7 +39,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0&quot;원&quot;"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="41">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -268,8 +269,17 @@
       <color rgb="00e40981"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A2744"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -326,6 +336,26 @@
         <fgColor rgb="00f5f5f7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A2744"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F4FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE7F3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -353,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -452,6 +482,31 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1312,10 +1367,10 @@
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="A30:C30"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId1"/>
@@ -6816,6 +6871,1513 @@
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E66"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>🎁 봉이 사은품 정책 카탈로그 (총 63개 상품)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="55" t="inlineStr">
+        <is>
+          <t>통신사</t>
+        </is>
+      </c>
+      <c r="C3" s="55" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="D3" s="55" t="inlineStr">
+        <is>
+          <t>상품 구성</t>
+        </is>
+      </c>
+      <c r="E3" s="55" t="inlineStr">
+        <is>
+          <t>사은품(원)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C4" s="56" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="n">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D5" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M</t>
+        </is>
+      </c>
+      <c r="E5" s="58" t="n">
+        <v>170000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="56" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C6" s="56" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G</t>
+        </is>
+      </c>
+      <c r="E6" s="58" t="n">
+        <v>170000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="56" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C7" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D7" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 이코노미</t>
+        </is>
+      </c>
+      <c r="E7" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C8" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 스탠다드</t>
+        </is>
+      </c>
+      <c r="E8" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="56" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D9" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 올</t>
+        </is>
+      </c>
+      <c r="E9" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="56" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C10" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 스탠다드 플러스</t>
+        </is>
+      </c>
+      <c r="E10" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="56" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D11" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 올 플러스</t>
+        </is>
+      </c>
+      <c r="E11" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 스탠다드 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E12" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D13" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 올 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E13" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C14" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D14" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 스탠다드 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E14" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C15" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D15" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 100M + B tv 올 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E15" s="58" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C16" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D16" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 이코노미</t>
+        </is>
+      </c>
+      <c r="E16" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C17" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D17" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 스탠다드</t>
+        </is>
+      </c>
+      <c r="E17" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D18" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 올</t>
+        </is>
+      </c>
+      <c r="E18" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C19" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D19" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 스탠다드 플러스</t>
+        </is>
+      </c>
+      <c r="E19" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C20" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D20" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 올 플러스</t>
+        </is>
+      </c>
+      <c r="E20" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D21" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 스탠다드 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E21" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C22" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 올 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E22" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D23" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 스탠다드 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E23" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D24" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 500M + B tv 올 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E24" s="58" t="n">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D25" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 이코노미</t>
+        </is>
+      </c>
+      <c r="E25" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C26" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D26" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 스탠다드</t>
+        </is>
+      </c>
+      <c r="E26" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C27" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D27" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 올</t>
+        </is>
+      </c>
+      <c r="E27" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C28" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D28" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 스탠다드 플러스</t>
+        </is>
+      </c>
+      <c r="E28" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C29" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D29" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 올 플러스</t>
+        </is>
+      </c>
+      <c r="E29" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="56" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C30" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D30" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 스탠다드 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E30" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C31" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D31" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 올 넷플릭스</t>
+        </is>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C32" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D32" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 스탠다드 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E32" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="56" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="56" t="inlineStr">
+        <is>
+          <t>SKT</t>
+        </is>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D33" s="57" t="inlineStr">
+        <is>
+          <t>인터넷 1G + B tv 올 넷플릭스 프리미엄</t>
+        </is>
+      </c>
+      <c r="E33" s="58" t="n">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="59" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D34" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M</t>
+        </is>
+      </c>
+      <c r="E34" s="61" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="59" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D35" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="n">
+        <v>140000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="59" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C36" s="59" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D36" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G</t>
+        </is>
+      </c>
+      <c r="E36" s="61" t="n">
+        <v>140000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="59" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C37" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D37" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M + 지니TV 베이직</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="n">
+        <v>370000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C38" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D38" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M + 지니TV 라이트</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="n">
+        <v>370000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="59" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C39" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D39" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M + 지니TV 에센스</t>
+        </is>
+      </c>
+      <c r="E39" s="61" t="n">
+        <v>370000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="59" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C40" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D40" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M + 지니TV 모든G</t>
+        </is>
+      </c>
+      <c r="E40" s="61" t="n">
+        <v>370000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C41" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D41" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 100M + 지니TV 디즈니+모든G</t>
+        </is>
+      </c>
+      <c r="E41" s="61" t="n">
+        <v>370000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="59" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C42" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D42" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M + 지니TV 베이직</t>
+        </is>
+      </c>
+      <c r="E42" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="59" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D43" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M + 지니TV 라이트</t>
+        </is>
+      </c>
+      <c r="E43" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C44" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D44" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M + 지니TV 에센스</t>
+        </is>
+      </c>
+      <c r="E44" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="59" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C45" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D45" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M + 지니TV 모든G</t>
+        </is>
+      </c>
+      <c r="E45" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="59" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C46" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D46" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 500M + 지니TV 디즈니+모든G</t>
+        </is>
+      </c>
+      <c r="E46" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="59" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C47" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D47" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G + 지니TV 베이직</t>
+        </is>
+      </c>
+      <c r="E47" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="59" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C48" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D48" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G + 지니TV 라이트</t>
+        </is>
+      </c>
+      <c r="E48" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="59" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C49" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D49" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G + 지니TV 에센스</t>
+        </is>
+      </c>
+      <c r="E49" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="59" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C50" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D50" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G + 지니TV 모든G</t>
+        </is>
+      </c>
+      <c r="E50" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="59" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="59" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C51" s="59" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D51" s="60" t="inlineStr">
+        <is>
+          <t>인터넷 1G + 지니TV 디즈니+모든G</t>
+        </is>
+      </c>
+      <c r="E51" s="61" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="62" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C52" s="62" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D52" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 100M</t>
+        </is>
+      </c>
+      <c r="E52" s="64" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="62" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C53" s="62" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D53" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 500M</t>
+        </is>
+      </c>
+      <c r="E53" s="64" t="n">
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="62" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C54" s="62" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="D54" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 1G</t>
+        </is>
+      </c>
+      <c r="E54" s="64" t="n">
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="62" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C55" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D55" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 100M + U+tv 실속형</t>
+        </is>
+      </c>
+      <c r="E55" s="64" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="62" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C56" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D56" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 100M + U+tv 기본형</t>
+        </is>
+      </c>
+      <c r="E56" s="64" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="62" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C57" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D57" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 100M + U+tv 프리미엄</t>
+        </is>
+      </c>
+      <c r="E57" s="64" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="62" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C58" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D58" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 100M + U+tv 프리미엄 VOD</t>
+        </is>
+      </c>
+      <c r="E58" s="64" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="62" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C59" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D59" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 500M + U+tv 실속형</t>
+        </is>
+      </c>
+      <c r="E59" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="62" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C60" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D60" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 500M + U+tv 기본형</t>
+        </is>
+      </c>
+      <c r="E60" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="62" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C61" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D61" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 500M + U+tv 프리미엄</t>
+        </is>
+      </c>
+      <c r="E61" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="62" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C62" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D62" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 500M + U+tv 프리미엄 VOD</t>
+        </is>
+      </c>
+      <c r="E62" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C63" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D63" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 1G + U+tv 실속형</t>
+        </is>
+      </c>
+      <c r="E63" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C64" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D64" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 1G + U+tv 기본형</t>
+        </is>
+      </c>
+      <c r="E64" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="62" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C65" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D65" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 1G + U+tv 프리미엄</t>
+        </is>
+      </c>
+      <c r="E65" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="62" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="62" t="inlineStr">
+        <is>
+          <t>LG U+</t>
+        </is>
+      </c>
+      <c r="C66" s="62" t="inlineStr">
+        <is>
+          <t>결합</t>
+        </is>
+      </c>
+      <c r="D66" s="63" t="inlineStr">
+        <is>
+          <t>인터넷 1G + U+tv 프리미엄 VOD</t>
+        </is>
+      </c>
+      <c r="E66" s="64" t="n">
+        <v>470000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>